<commit_message>
Short import template: 8 columns each for patients and doctors
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRRBvkKjt3A9PgQv7tKcVq
</commit_message>
<xml_diff>
--- a/project/sample-imports/doctors-uat.xlsx
+++ b/project/sample-imports/doctors-uat.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="45">
   <si>
     <t>staff_number</t>
   </si>
@@ -37,27 +37,6 @@
     <t>role</t>
   </si>
   <si>
-    <t>department</t>
-  </si>
-  <si>
-    <t>qualifications</t>
-  </si>
-  <si>
-    <t>languages</t>
-  </si>
-  <si>
-    <t>years_experience</t>
-  </si>
-  <si>
-    <t>shift_start</t>
-  </si>
-  <si>
-    <t>shift_end</t>
-  </si>
-  <si>
-    <t>shift_days</t>
-  </si>
-  <si>
     <t>UAT-D-01</t>
   </si>
   <si>
@@ -82,27 +61,6 @@
     <t>doctor</t>
   </si>
   <si>
-    <t>General Medicine</t>
-  </si>
-  <si>
-    <t>MBChB;DipPEC</t>
-  </si>
-  <si>
-    <t>English;isiZulu</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>08:00</t>
-  </si>
-  <si>
-    <t>16:00</t>
-  </si>
-  <si>
-    <t>Mon;Tue;Wed;Thu;Fri</t>
-  </si>
-  <si>
     <t>UAT-D-02</t>
   </si>
   <si>
@@ -124,27 +82,6 @@
     <t>Cardiologist</t>
   </si>
   <si>
-    <t>Cardiology</t>
-  </si>
-  <si>
-    <t>MBChB;MMed Internal Medicine;FCP(SA)</t>
-  </si>
-  <si>
-    <t>English;Sesotho;Afrikaans</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>07:00</t>
-  </si>
-  <si>
-    <t>15:00</t>
-  </si>
-  <si>
-    <t>Mon;Wed;Fri</t>
-  </si>
-  <si>
     <t>UAT-D-03</t>
   </si>
   <si>
@@ -166,27 +103,6 @@
     <t>Paediatrician</t>
   </si>
   <si>
-    <t>Paediatrics</t>
-  </si>
-  <si>
-    <t>MBChB;DCH(SA);MMed Paediatrics</t>
-  </si>
-  <si>
-    <t>English;Afrikaans</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>09:00</t>
-  </si>
-  <si>
-    <t>17:00</t>
-  </si>
-  <si>
-    <t>Tue;Wed;Thu;Sat</t>
-  </si>
-  <si>
     <t>UAT-D-04</t>
   </si>
   <si>
@@ -208,27 +124,6 @@
     <t>Dermatologist</t>
   </si>
   <si>
-    <t>Dermatology</t>
-  </si>
-  <si>
-    <t>MBChB;FC Derm(SA)</t>
-  </si>
-  <si>
-    <t>English;isiXhosa;Setswana</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>10:00</t>
-  </si>
-  <si>
-    <t>18:00</t>
-  </si>
-  <si>
-    <t>Mon;Tue;Thu;Fri</t>
-  </si>
-  <si>
     <t>UAT-D-05</t>
   </si>
   <si>
@@ -251,24 +146,6 @@
   </si>
   <si>
     <t>nurse</t>
-  </si>
-  <si>
-    <t>Emergency</t>
-  </si>
-  <si>
-    <t>BCur;Diploma Emergency Nursing</t>
-  </si>
-  <si>
-    <t>English;isiZulu;Siswati</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>23:00</t>
-  </si>
-  <si>
-    <t>Fri;Sat;Sun</t>
   </si>
 </sst>
 </file>
@@ -645,10 +522,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -673,261 +550,135 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="C2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="D2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="E2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="F2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="G2" t="s">
         <v>14</v>
       </c>
+      <c r="H2" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" t="s">
         <v>15</v>
       </c>
-      <c r="B2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I2" t="s">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>23</v>
       </c>
-      <c r="J2" t="s">
+      <c r="B4" t="s">
         <v>24</v>
       </c>
-      <c r="K2" t="s">
+      <c r="C4" t="s">
         <v>25</v>
       </c>
-      <c r="L2" t="s">
+      <c r="D4" t="s">
         <v>26</v>
       </c>
-      <c r="M2" t="s">
+      <c r="E4" t="s">
         <v>27</v>
       </c>
-      <c r="N2" t="s">
+      <c r="F4" t="s">
         <v>28</v>
       </c>
-      <c r="O2" t="s">
+      <c r="G4" t="s">
         <v>29</v>
       </c>
+      <c r="H4" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>30</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B5" t="s">
         <v>31</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C5" t="s">
         <v>32</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D5" t="s">
         <v>33</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E5" t="s">
         <v>34</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F5" t="s">
         <v>35</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G5" t="s">
         <v>36</v>
       </c>
-      <c r="H3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I3" t="s">
+      <c r="H5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>37</v>
       </c>
-      <c r="J3" t="s">
+      <c r="B6" t="s">
         <v>38</v>
       </c>
-      <c r="K3" t="s">
+      <c r="C6" t="s">
         <v>39</v>
       </c>
-      <c r="L3" t="s">
+      <c r="D6" t="s">
         <v>40</v>
       </c>
-      <c r="M3" t="s">
+      <c r="E6" t="s">
         <v>41</v>
       </c>
-      <c r="N3" t="s">
+      <c r="F6" t="s">
         <v>42</v>
       </c>
-      <c r="O3" t="s">
+      <c r="G6" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="H6" t="s">
         <v>44</v>
-      </c>
-      <c r="B4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" t="s">
-        <v>47</v>
-      </c>
-      <c r="E4" t="s">
-        <v>48</v>
-      </c>
-      <c r="F4" t="s">
-        <v>49</v>
-      </c>
-      <c r="G4" t="s">
-        <v>50</v>
-      </c>
-      <c r="H4" t="s">
-        <v>22</v>
-      </c>
-      <c r="I4" t="s">
-        <v>51</v>
-      </c>
-      <c r="J4" t="s">
-        <v>52</v>
-      </c>
-      <c r="K4" t="s">
-        <v>53</v>
-      </c>
-      <c r="L4" t="s">
-        <v>54</v>
-      </c>
-      <c r="M4" t="s">
-        <v>55</v>
-      </c>
-      <c r="N4" t="s">
-        <v>56</v>
-      </c>
-      <c r="O4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>58</v>
-      </c>
-      <c r="B5" t="s">
-        <v>59</v>
-      </c>
-      <c r="C5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D5" t="s">
-        <v>61</v>
-      </c>
-      <c r="E5" t="s">
-        <v>62</v>
-      </c>
-      <c r="F5" t="s">
-        <v>63</v>
-      </c>
-      <c r="G5" t="s">
-        <v>64</v>
-      </c>
-      <c r="H5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I5" t="s">
-        <v>65</v>
-      </c>
-      <c r="J5" t="s">
-        <v>66</v>
-      </c>
-      <c r="K5" t="s">
-        <v>67</v>
-      </c>
-      <c r="L5" t="s">
-        <v>68</v>
-      </c>
-      <c r="M5" t="s">
-        <v>69</v>
-      </c>
-      <c r="N5" t="s">
-        <v>70</v>
-      </c>
-      <c r="O5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>72</v>
-      </c>
-      <c r="B6" t="s">
-        <v>73</v>
-      </c>
-      <c r="C6" t="s">
-        <v>74</v>
-      </c>
-      <c r="D6" t="s">
-        <v>75</v>
-      </c>
-      <c r="E6" t="s">
-        <v>76</v>
-      </c>
-      <c r="F6" t="s">
-        <v>77</v>
-      </c>
-      <c r="G6" t="s">
-        <v>78</v>
-      </c>
-      <c r="H6" t="s">
-        <v>79</v>
-      </c>
-      <c r="I6" t="s">
-        <v>80</v>
-      </c>
-      <c r="J6" t="s">
-        <v>81</v>
-      </c>
-      <c r="K6" t="s">
-        <v>82</v>
-      </c>
-      <c r="L6" t="s">
-        <v>83</v>
-      </c>
-      <c r="M6" t="s">
-        <v>70</v>
-      </c>
-      <c r="N6" t="s">
-        <v>84</v>
-      </c>
-      <c r="O6" t="s">
-        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>